<commit_message>
Apply on VO by Youth and upload images in gallery image by youth
</commit_message>
<xml_diff>
--- a/src/main/resources/UserDetails.xlsx
+++ b/src/main/resources/UserDetails.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2448" windowWidth="17856" windowHeight="4272"/>
+    <workbookView xWindow="0" yWindow="2448" windowWidth="17856" windowHeight="5448"/>
   </bookViews>
   <sheets>
     <sheet name="UserData" sheetId="1" r:id="rId1"/>
@@ -15,79 +15,21 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>Email</t>
   </si>
   <si>
-    <t>AndreeQuigley@yopmail.com</t>
+    <t>JodiMcDermott@yopmail.com</t>
   </si>
   <si>
-    <t>MartaPagac@yopmail.com</t>
-  </si>
-  <si>
-    <t>VenusWunsch@yopmail.com</t>
-  </si>
-  <si>
-    <t>MarcCrooks@yopmail.com</t>
-  </si>
-  <si>
-    <t>HaileyWaters@yopmail.com</t>
-  </si>
-  <si>
-    <t>KaronStroman@yopmail.com</t>
-  </si>
-  <si>
-    <t>BradleyTorp@yopmail.com</t>
-  </si>
-  <si>
-    <t>MrLynetteGlover@yopmail.com</t>
-  </si>
-  <si>
-    <t>CarrollSchroeder@yopmail.com</t>
-  </si>
-  <si>
-    <t>MrLindseyReichel@yopmail.com</t>
-  </si>
-  <si>
-    <t>StaceyBeier@yopmail.com</t>
-  </si>
-  <si>
-    <t>DwainWisoky@yopmail.com</t>
-  </si>
-  <si>
-    <t>DustinKulas@yopmail.com</t>
-  </si>
-  <si>
-    <t>VincentConnelly@yopmail.com</t>
-  </si>
-  <si>
-    <t>LucasWhite@yopmail.com</t>
-  </si>
-  <si>
-    <t>HoytRauIII@yopmail.com</t>
-  </si>
-  <si>
-    <t>DennisMarvin@yopmail.com</t>
-  </si>
-  <si>
-    <t>EdmundBoyle@yopmail.com</t>
-  </si>
-  <si>
-    <t>DanielLarson@yopmail.com</t>
-  </si>
-  <si>
-    <t>MsBretPurdy@yopmail.com</t>
-  </si>
-  <si>
-    <t>LidiaBarrows@yopmail.com</t>
+    <t>AlecLang@yopmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -420,134 +362,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A30"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" customWidth="true" width="42.88671875"/>
-    <col min="2" max="2" customWidth="true" width="25.88671875"/>
-    <col min="3" max="3" customWidth="true" width="30.88671875"/>
-    <col min="4" max="4" customWidth="true" width="30.21875"/>
-    <col min="5" max="5" customWidth="true" width="22.44140625"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A1" t="s" s="0">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A3" t="s" s="0">
+      <c r="A3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" t="s" s="0">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A5" t="s" s="0">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A6" t="s" s="0">
-        <v>5</v>
-      </c>
-    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3"/>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3"/>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3"/>
     <row r="8" spans="1:1" x14ac:dyDescent="0.3"/>
     <row r="9" spans="1:1" x14ac:dyDescent="0.3"/>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.3"/>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.3"/>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.3"/>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.3"/>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.3"/>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A15" t="s" s="0">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A16" t="s" s="0">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A17" t="s" s="0">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A18" t="s" s="0">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A19" t="s" s="0">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A20" t="s" s="0">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A21" t="s" s="0">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A22" t="s" s="0">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A23" t="s" s="0">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="s" s="0">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="s" s="0">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="s" s="0">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="s" s="0">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="s" s="0">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="s" s="0">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="s" s="0">
-        <v>21</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>